<commit_message>
moved transmission from electricity to final electricity in neverland example
</commit_message>
<xml_diff>
--- a/hypatia/examples/Neverland/config.xlsx
+++ b/hypatia/examples/Neverland/config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10394890_polimi_it/Documents/Research/Repositories/Hypatia-polimi/hypatia/examples/Neverland/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="11_0F3735819E76DBB756A3AF6C12E22BFD38F29026" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5771E7E-4490-4EAA-B4DC-5E5E580F7531}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="11_0F3735819E76DBB756A3AF6C12E22BFD38F29026" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E5CA85F-52E2-4031-9E57-BF6D5972283E}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Techs" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="68">
   <si>
     <t>Technology</t>
   </si>
@@ -191,12 +191,6 @@
     <t>#f76ffc</t>
   </si>
   <si>
-    <t>Resource</t>
-  </si>
-  <si>
-    <t>Demand</t>
-  </si>
-  <si>
     <t>#000000</t>
   </si>
   <si>
@@ -215,9 +209,6 @@
     <t>Supply</t>
   </si>
   <si>
-    <t>Transmission</t>
-  </si>
-  <si>
     <t>#080808</t>
   </si>
   <si>
@@ -231,6 +222,12 @@
   </si>
   <si>
     <t>Electricity</t>
+  </si>
+  <si>
+    <t>Power Transmission</t>
+  </si>
+  <si>
+    <t>Power Demand</t>
   </si>
 </sst>
 </file>
@@ -629,10 +626,10 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E2" t="s">
         <v>7</v>
@@ -649,10 +646,10 @@
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E3" t="s">
         <v>7</v>
@@ -669,10 +666,10 @@
         <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E4" t="s">
         <v>12</v>
@@ -689,10 +686,10 @@
         <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E5" t="s">
         <v>12</v>
@@ -709,10 +706,10 @@
         <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D6" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E6" t="s">
         <v>12</v>
@@ -729,10 +726,10 @@
         <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D7" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E7" t="s">
         <v>12</v>
@@ -749,10 +746,10 @@
         <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E8" t="s">
         <v>12</v>
@@ -769,10 +766,10 @@
         <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="D9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E9" t="s">
         <v>12</v>
@@ -886,10 +883,10 @@
         <v>34</v>
       </c>
       <c r="C2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" t="s">
         <v>55</v>
-      </c>
-      <c r="D2" t="s">
-        <v>57</v>
       </c>
       <c r="E2" t="s">
         <v>8</v>
@@ -903,10 +900,10 @@
         <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E3" t="s">
         <v>10</v>
@@ -920,10 +917,10 @@
         <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E4" t="s">
         <v>13</v>
@@ -937,10 +934,10 @@
         <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E5" t="s">
         <v>13</v>
@@ -978,7 +975,7 @@
         <v>42</v>
       </c>
       <c r="C2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -989,7 +986,7 @@
         <v>44</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>